<commit_message>
:hibiscus: CCA run with final data (for D2 -> 5000 randomized matrix instead of 1000)
</commit_message>
<xml_diff>
--- a/data/derived_data/6_NMI_CCA/Dataset_1/CCA_CONFIGS_ITS_D1_04.xlsx
+++ b/data/derived_data/6_NMI_CCA/Dataset_1/CCA_CONFIGS_ITS_D1_04.xlsx
@@ -425,7 +425,7 @@
         <v>0.0001</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9994</v>
+        <v>0.9979</v>
       </c>
     </row>
     <row r="3">
@@ -436,16 +436,16 @@
         <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>0.538286356209151</v>
+        <v>0.538286356209148</v>
       </c>
       <c r="D3" t="n">
-        <v>4.50941525971249</v>
+        <v>4.50941525971246</v>
       </c>
       <c r="E3" t="n">
         <v>0.0001</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8826</v>
+        <v>0.8595</v>
       </c>
     </row>
     <row r="4">
@@ -465,7 +465,7 @@
         <v>0.0001</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9962</v>
+        <v>0.9955</v>
       </c>
     </row>
     <row r="5">
@@ -485,7 +485,7 @@
         <v>0.0001</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9968</v>
+        <v>0.9978</v>
       </c>
     </row>
     <row r="6">
@@ -505,7 +505,7 @@
         <v>0.0001</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9021</v>
+        <v>0.8847</v>
       </c>
     </row>
   </sheetData>

</xml_diff>